<commit_message>
25 May 2026 - Sync
</commit_message>
<xml_diff>
--- a/Import_WD.xlsx
+++ b/Import_WD.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ichorsystems-my.sharepoint.com/personal/kmageshkumar_ichorsystems_com/Documents/Scripts/WD Create FBDI/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="44" documentId="13_ncr:1_{1448A942-2B91-453D-A348-8841A73FF17B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0F2EF7A7-2A08-4F36-A7FB-99A40FD26A2C}"/>
+  <xr:revisionPtr revIDLastSave="53" documentId="13_ncr:1_{1448A942-2B91-453D-A348-8841A73FF17B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EE72D69D-DBB0-477B-8ACF-9DFE0AA890DA}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="180" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="210" uniqueCount="103">
   <si>
     <t>WD Number</t>
   </si>
@@ -245,58 +245,106 @@
     <t>SGP_TEMPLATE_LAM_AFVI2_JTS</t>
   </si>
   <si>
-    <t>437388R03-XXT-GPA</t>
-  </si>
-  <si>
-    <t>437388R03-XXT-GPB</t>
-  </si>
-  <si>
-    <t>437388R03-XXT-GPC</t>
-  </si>
-  <si>
-    <t>511956-DG-GPA</t>
-  </si>
-  <si>
-    <t>511956-DG-GPB</t>
-  </si>
-  <si>
-    <t>511956-DG-GPC</t>
-  </si>
-  <si>
-    <t>701530R05-KA-GP</t>
-  </si>
-  <si>
-    <t>709451-XG3T-GPLL</t>
-  </si>
-  <si>
-    <t>709453-XG3T-GPLL</t>
-  </si>
-  <si>
-    <t>709726-XG3T-GPLL</t>
-  </si>
-  <si>
-    <t>709727-XG3T-GPLL</t>
-  </si>
-  <si>
-    <t>709837-XA3T-GPA</t>
-  </si>
-  <si>
-    <t>709837-XA3T-GPB</t>
-  </si>
-  <si>
-    <t>709837-XA3T-GPC</t>
-  </si>
-  <si>
-    <t>709839-XA3T-SLD</t>
-  </si>
-  <si>
-    <t>C01340R1-EY3-GP2A</t>
-  </si>
-  <si>
-    <t>C01340R1-EY3-GP2B</t>
-  </si>
-  <si>
-    <t>C01340R1-EY3-GP2C</t>
+    <t>SGP_TEMPLATE_NSO_1_STICK</t>
+  </si>
+  <si>
+    <t>500678N15-DX-GPB</t>
+  </si>
+  <si>
+    <t>500678N15-DX-GPC</t>
+  </si>
+  <si>
+    <t>500678N15-DX-GPE</t>
+  </si>
+  <si>
+    <t>500678N15-DX-GPF</t>
+  </si>
+  <si>
+    <t>500678N15-DX-GPG</t>
+  </si>
+  <si>
+    <t>510107N01-DG-GPB</t>
+  </si>
+  <si>
+    <t>511073-DG-GPA</t>
+  </si>
+  <si>
+    <t>511073-DG-GPB</t>
+  </si>
+  <si>
+    <t>511073-DG-GPC</t>
+  </si>
+  <si>
+    <t>511401-DF-GP</t>
+  </si>
+  <si>
+    <t>511766-DF-GPA</t>
+  </si>
+  <si>
+    <t>511766-DF-GPB</t>
+  </si>
+  <si>
+    <t>511766-DF-GPC</t>
+  </si>
+  <si>
+    <t>512032-DF-GPA</t>
+  </si>
+  <si>
+    <t>512032-DF-GPB</t>
+  </si>
+  <si>
+    <t>512032-DF-GPC</t>
+  </si>
+  <si>
+    <t>512266-DG-GPA</t>
+  </si>
+  <si>
+    <t>512266-DG-GPB</t>
+  </si>
+  <si>
+    <t>512266-DG-GPC</t>
+  </si>
+  <si>
+    <t>512266-DG-INZC</t>
+  </si>
+  <si>
+    <t>512492-DF-GP</t>
+  </si>
+  <si>
+    <t>512498-DF-GPA</t>
+  </si>
+  <si>
+    <t>512498-DF-GPB</t>
+  </si>
+  <si>
+    <t>512498-DF-GPC</t>
+  </si>
+  <si>
+    <t>512597-DF-GPA</t>
+  </si>
+  <si>
+    <t>512597-DF-GPB</t>
+  </si>
+  <si>
+    <t>512597-DF-GPC</t>
+  </si>
+  <si>
+    <t>709190-XA3T-SLD</t>
+  </si>
+  <si>
+    <t>709612-XA3T-SLD</t>
+  </si>
+  <si>
+    <t>710287-XA3T-GPA</t>
+  </si>
+  <si>
+    <t>710287-XA3T-GPB</t>
+  </si>
+  <si>
+    <t>710287-XA3T-GPC</t>
+  </si>
+  <si>
+    <t>710287-XA3T-SLD</t>
   </si>
 </sst>
 </file>
@@ -385,10 +433,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -695,11 +739,11 @@
       </c>
     </row>
     <row r="2" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A2" s="5" t="s">
-        <v>69</v>
-      </c>
-      <c r="B2" s="5" t="s">
-        <v>34</v>
+      <c r="A2" t="s">
+        <v>70</v>
+      </c>
+      <c r="B2" t="s">
+        <v>24</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>64</v>
@@ -719,11 +763,11 @@
       </c>
     </row>
     <row r="3" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A3" s="5" t="s">
-        <v>70</v>
-      </c>
-      <c r="B3" s="5" t="s">
-        <v>34</v>
+      <c r="A3" t="s">
+        <v>71</v>
+      </c>
+      <c r="B3" t="s">
+        <v>24</v>
       </c>
       <c r="D3" s="1" t="s">
         <v>64</v>
@@ -741,11 +785,11 @@
       <c r="I3" s="1"/>
     </row>
     <row r="4" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A4" s="5" t="s">
-        <v>71</v>
-      </c>
-      <c r="B4" s="5" t="s">
-        <v>34</v>
+      <c r="A4" t="s">
+        <v>72</v>
+      </c>
+      <c r="B4" t="s">
+        <v>24</v>
       </c>
       <c r="D4" s="1" t="s">
         <v>64</v>
@@ -765,11 +809,11 @@
       </c>
     </row>
     <row r="5" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A5" s="5" t="s">
-        <v>72</v>
-      </c>
-      <c r="B5" s="5" t="s">
-        <v>9</v>
+      <c r="A5" t="s">
+        <v>73</v>
+      </c>
+      <c r="B5" t="s">
+        <v>24</v>
       </c>
       <c r="D5" s="1" t="s">
         <v>64</v>
@@ -792,11 +836,11 @@
       </c>
     </row>
     <row r="6" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A6" s="5" t="s">
-        <v>73</v>
-      </c>
-      <c r="B6" s="5" t="s">
-        <v>9</v>
+      <c r="A6" t="s">
+        <v>74</v>
+      </c>
+      <c r="B6" t="s">
+        <v>24</v>
       </c>
       <c r="D6" s="1" t="s">
         <v>64</v>
@@ -816,11 +860,11 @@
       </c>
     </row>
     <row r="7" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A7" s="5" t="s">
-        <v>74</v>
-      </c>
-      <c r="B7" s="5" t="s">
-        <v>9</v>
+      <c r="A7" t="s">
+        <v>75</v>
+      </c>
+      <c r="B7" t="s">
+        <v>69</v>
       </c>
       <c r="D7" s="1" t="s">
         <v>64</v>
@@ -840,11 +884,11 @@
       </c>
     </row>
     <row r="8" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A8" s="5" t="s">
-        <v>75</v>
-      </c>
-      <c r="B8" s="5" t="s">
-        <v>34</v>
+      <c r="A8" t="s">
+        <v>76</v>
+      </c>
+      <c r="B8" t="s">
+        <v>10</v>
       </c>
       <c r="D8" s="1" t="s">
         <v>64</v>
@@ -864,11 +908,11 @@
       </c>
     </row>
     <row r="9" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A9" s="5" t="s">
-        <v>76</v>
-      </c>
-      <c r="B9" s="5" t="s">
-        <v>32</v>
+      <c r="A9" t="s">
+        <v>77</v>
+      </c>
+      <c r="B9" t="s">
+        <v>10</v>
       </c>
       <c r="D9" s="1" t="s">
         <v>64</v>
@@ -886,11 +930,11 @@
       <c r="I9" s="1"/>
     </row>
     <row r="10" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A10" s="5" t="s">
-        <v>77</v>
-      </c>
-      <c r="B10" s="5" t="s">
-        <v>32</v>
+      <c r="A10" t="s">
+        <v>78</v>
+      </c>
+      <c r="B10" t="s">
+        <v>10</v>
       </c>
       <c r="D10" s="1" t="s">
         <v>64</v>
@@ -908,11 +952,11 @@
       <c r="I10" s="1"/>
     </row>
     <row r="11" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A11" s="5" t="s">
-        <v>78</v>
-      </c>
-      <c r="B11" s="5" t="s">
-        <v>32</v>
+      <c r="A11" t="s">
+        <v>79</v>
+      </c>
+      <c r="B11" t="s">
+        <v>16</v>
       </c>
       <c r="D11" s="1" t="s">
         <v>64</v>
@@ -930,11 +974,11 @@
       <c r="I11" s="1"/>
     </row>
     <row r="12" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A12" s="5" t="s">
-        <v>79</v>
-      </c>
-      <c r="B12" s="5" t="s">
-        <v>32</v>
+      <c r="A12" t="s">
+        <v>80</v>
+      </c>
+      <c r="B12" t="s">
+        <v>12</v>
       </c>
       <c r="D12" s="1" t="s">
         <v>64</v>
@@ -954,11 +998,11 @@
       </c>
     </row>
     <row r="13" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A13" s="5" t="s">
-        <v>80</v>
-      </c>
-      <c r="B13" s="5" t="s">
-        <v>29</v>
+      <c r="A13" t="s">
+        <v>81</v>
+      </c>
+      <c r="B13" t="s">
+        <v>12</v>
       </c>
       <c r="D13" s="1" t="s">
         <v>64</v>
@@ -976,11 +1020,11 @@
       <c r="I13" s="1"/>
     </row>
     <row r="14" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A14" s="5" t="s">
-        <v>81</v>
-      </c>
-      <c r="B14" s="5" t="s">
-        <v>29</v>
+      <c r="A14" t="s">
+        <v>82</v>
+      </c>
+      <c r="B14" t="s">
+        <v>12</v>
       </c>
       <c r="D14" s="1" t="s">
         <v>64</v>
@@ -998,11 +1042,11 @@
       <c r="I14" s="1"/>
     </row>
     <row r="15" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A15" s="5" t="s">
-        <v>82</v>
-      </c>
-      <c r="B15" s="5" t="s">
-        <v>29</v>
+      <c r="A15" t="s">
+        <v>83</v>
+      </c>
+      <c r="B15" t="s">
+        <v>12</v>
       </c>
       <c r="D15" s="1" t="s">
         <v>64</v>
@@ -1020,11 +1064,11 @@
       <c r="I15" s="1"/>
     </row>
     <row r="16" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A16" s="5" t="s">
-        <v>83</v>
-      </c>
-      <c r="B16" s="5" t="s">
-        <v>23</v>
+      <c r="A16" t="s">
+        <v>84</v>
+      </c>
+      <c r="B16" t="s">
+        <v>12</v>
       </c>
       <c r="D16" s="1" t="s">
         <v>64</v>
@@ -1042,11 +1086,11 @@
       <c r="I16" s="1"/>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A17" s="5" t="s">
-        <v>84</v>
-      </c>
-      <c r="B17" s="5" t="s">
-        <v>34</v>
+      <c r="A17" t="s">
+        <v>85</v>
+      </c>
+      <c r="B17" t="s">
+        <v>12</v>
       </c>
       <c r="D17" s="1" t="s">
         <v>64</v>
@@ -1064,11 +1108,11 @@
       <c r="I17" s="1"/>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A18" s="5" t="s">
-        <v>85</v>
-      </c>
-      <c r="B18" s="5" t="s">
-        <v>34</v>
+      <c r="A18" t="s">
+        <v>86</v>
+      </c>
+      <c r="B18" t="s">
+        <v>10</v>
       </c>
       <c r="D18" s="1" t="s">
         <v>64</v>
@@ -1086,11 +1130,11 @@
       <c r="I18" s="1"/>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A19" s="5" t="s">
-        <v>86</v>
-      </c>
-      <c r="B19" s="5" t="s">
-        <v>34</v>
+      <c r="A19" t="s">
+        <v>87</v>
+      </c>
+      <c r="B19" t="s">
+        <v>10</v>
       </c>
       <c r="D19" s="1" t="s">
         <v>64</v>
@@ -1110,6 +1154,12 @@
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>88</v>
+      </c>
+      <c r="B20" t="s">
+        <v>10</v>
+      </c>
       <c r="D20" s="1" t="s">
         <v>64</v>
       </c>
@@ -1128,6 +1178,12 @@
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>89</v>
+      </c>
+      <c r="B21" t="s">
+        <v>8</v>
+      </c>
       <c r="D21" s="1" t="s">
         <v>64</v>
       </c>
@@ -1144,6 +1200,12 @@
       <c r="I21" s="1"/>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>90</v>
+      </c>
+      <c r="B22" t="s">
+        <v>15</v>
+      </c>
       <c r="D22" s="1" t="s">
         <v>64</v>
       </c>
@@ -1162,6 +1224,12 @@
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>91</v>
+      </c>
+      <c r="B23" t="s">
+        <v>11</v>
+      </c>
       <c r="D23" s="1" t="s">
         <v>64</v>
       </c>
@@ -1180,6 +1248,12 @@
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>92</v>
+      </c>
+      <c r="B24" t="s">
+        <v>11</v>
+      </c>
       <c r="D24" s="1" t="s">
         <v>64</v>
       </c>
@@ -1196,6 +1270,12 @@
       <c r="I24" s="1"/>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>93</v>
+      </c>
+      <c r="B25" t="s">
+        <v>11</v>
+      </c>
       <c r="D25" s="1" t="s">
         <v>64</v>
       </c>
@@ -1214,6 +1294,12 @@
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>94</v>
+      </c>
+      <c r="B26" t="s">
+        <v>12</v>
+      </c>
       <c r="D26" s="1" t="s">
         <v>64</v>
       </c>
@@ -1232,7 +1318,12 @@
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A27" s="6"/>
+      <c r="A27" t="s">
+        <v>95</v>
+      </c>
+      <c r="B27" t="s">
+        <v>12</v>
+      </c>
       <c r="D27" s="1" t="s">
         <v>64</v>
       </c>
@@ -1251,6 +1342,12 @@
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>96</v>
+      </c>
+      <c r="B28" t="s">
+        <v>12</v>
+      </c>
       <c r="D28" s="1" t="s">
         <v>64</v>
       </c>
@@ -1267,6 +1364,12 @@
       <c r="I28" s="1"/>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>97</v>
+      </c>
+      <c r="B29" t="s">
+        <v>23</v>
+      </c>
       <c r="D29" s="1" t="s">
         <v>64</v>
       </c>
@@ -1285,6 +1388,12 @@
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>98</v>
+      </c>
+      <c r="B30" t="s">
+        <v>23</v>
+      </c>
       <c r="D30" s="1" t="s">
         <v>64</v>
       </c>
@@ -1301,6 +1410,12 @@
       <c r="I30" s="1"/>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>99</v>
+      </c>
+      <c r="B31" t="s">
+        <v>29</v>
+      </c>
       <c r="E31" s="2"/>
       <c r="G31" s="1" t="s">
         <v>4</v>
@@ -1311,6 +1426,12 @@
       <c r="I31" s="1"/>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>100</v>
+      </c>
+      <c r="B32" t="s">
+        <v>29</v>
+      </c>
       <c r="E32" s="2"/>
       <c r="G32" s="1" t="s">
         <v>4</v>
@@ -1320,19 +1441,35 @@
       </c>
       <c r="I32" s="1"/>
     </row>
-    <row r="44" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>101</v>
+      </c>
+      <c r="B33" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>102</v>
+      </c>
+      <c r="B34" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A44" s="6"/>
     </row>
-    <row r="45" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A45" s="6"/>
     </row>
-    <row r="46" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A46" s="6"/>
     </row>
-    <row r="47" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A47" s="6"/>
     </row>
-    <row r="48" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A48" s="6"/>
     </row>
     <row r="49" spans="1:1" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
24 Jul 2026 - Sync
</commit_message>
<xml_diff>
--- a/Import_WD.xlsx
+++ b/Import_WD.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ichorsystems-my.sharepoint.com/personal/kmageshkumar_ichorsystems_com/Documents/Scripts/WD Create FBDI/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="53" documentId="13_ncr:1_{1448A942-2B91-453D-A348-8841A73FF17B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EE72D69D-DBB0-477B-8ACF-9DFE0AA890DA}"/>
+  <xr:revisionPtr revIDLastSave="118" documentId="13_ncr:1_{1448A942-2B91-453D-A348-8841A73FF17B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{17C8CA57-6B38-4222-A65B-58993127ABE4}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="210" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="182" uniqueCount="91">
   <si>
     <t>WD Number</t>
   </si>
@@ -245,106 +245,70 @@
     <t>SGP_TEMPLATE_LAM_AFVI2_JTS</t>
   </si>
   <si>
+    <t>A04027-TY-GPA</t>
+  </si>
+  <si>
+    <t>SGP_TEMPLATE_DPN</t>
+  </si>
+  <si>
+    <t>A04027-TY-GPB</t>
+  </si>
+  <si>
+    <t>A04622-TY-GPC</t>
+  </si>
+  <si>
+    <t>A04622-TY-GPD</t>
+  </si>
+  <si>
+    <t>A04619-TY-GPA</t>
+  </si>
+  <si>
+    <t>A04619-TY-GPB</t>
+  </si>
+  <si>
+    <t>709850-XA3T-GPA</t>
+  </si>
+  <si>
+    <t>709850-XA3T-GPB</t>
+  </si>
+  <si>
+    <t>709850-XA3T-GPC</t>
+  </si>
+  <si>
+    <t>710366-XXT-GPA</t>
+  </si>
+  <si>
+    <t>SGP_TEMPLATE_NAPA</t>
+  </si>
+  <si>
+    <t>710366-XXT-GPB</t>
+  </si>
+  <si>
+    <t>710366-XXT-GPC</t>
+  </si>
+  <si>
+    <t>710411-XXT-GPA</t>
+  </si>
+  <si>
+    <t>710411-XXT-GPB</t>
+  </si>
+  <si>
+    <t>710411-XXT-GPC</t>
+  </si>
+  <si>
+    <t>A02651R2-TY-GPA</t>
+  </si>
+  <si>
     <t>SGP_TEMPLATE_NSO_1_STICK</t>
   </si>
   <si>
-    <t>500678N15-DX-GPB</t>
-  </si>
-  <si>
-    <t>500678N15-DX-GPC</t>
-  </si>
-  <si>
-    <t>500678N15-DX-GPE</t>
-  </si>
-  <si>
-    <t>500678N15-DX-GPF</t>
-  </si>
-  <si>
-    <t>500678N15-DX-GPG</t>
-  </si>
-  <si>
-    <t>510107N01-DG-GPB</t>
-  </si>
-  <si>
-    <t>511073-DG-GPA</t>
-  </si>
-  <si>
-    <t>511073-DG-GPB</t>
-  </si>
-  <si>
-    <t>511073-DG-GPC</t>
-  </si>
-  <si>
-    <t>511401-DF-GP</t>
-  </si>
-  <si>
-    <t>511766-DF-GPA</t>
-  </si>
-  <si>
-    <t>511766-DF-GPB</t>
-  </si>
-  <si>
-    <t>511766-DF-GPC</t>
-  </si>
-  <si>
-    <t>512032-DF-GPA</t>
-  </si>
-  <si>
-    <t>512032-DF-GPB</t>
-  </si>
-  <si>
-    <t>512032-DF-GPC</t>
-  </si>
-  <si>
-    <t>512266-DG-GPA</t>
-  </si>
-  <si>
-    <t>512266-DG-GPB</t>
-  </si>
-  <si>
-    <t>512266-DG-GPC</t>
-  </si>
-  <si>
-    <t>512266-DG-INZC</t>
-  </si>
-  <si>
-    <t>512492-DF-GP</t>
-  </si>
-  <si>
-    <t>512498-DF-GPA</t>
-  </si>
-  <si>
-    <t>512498-DF-GPB</t>
-  </si>
-  <si>
-    <t>512498-DF-GPC</t>
-  </si>
-  <si>
-    <t>512597-DF-GPA</t>
-  </si>
-  <si>
-    <t>512597-DF-GPB</t>
-  </si>
-  <si>
-    <t>512597-DF-GPC</t>
-  </si>
-  <si>
-    <t>709190-XA3T-SLD</t>
-  </si>
-  <si>
-    <t>709612-XA3T-SLD</t>
-  </si>
-  <si>
-    <t>710287-XA3T-GPA</t>
-  </si>
-  <si>
-    <t>710287-XA3T-GPB</t>
-  </si>
-  <si>
-    <t>710287-XA3T-GPC</t>
-  </si>
-  <si>
-    <t>710287-XA3T-SLD</t>
+    <t>A02651R2-TY-GPD</t>
+  </si>
+  <si>
+    <t>C02371-EY2-GP1</t>
+  </si>
+  <si>
+    <t>C02371-EY2-GP2</t>
   </si>
 </sst>
 </file>
@@ -740,10 +704,10 @@
     </row>
     <row r="2" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="B2" t="s">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>64</v>
@@ -764,10 +728,10 @@
     </row>
     <row r="3" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="B3" t="s">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="D3" s="1" t="s">
         <v>64</v>
@@ -786,10 +750,10 @@
     </row>
     <row r="4" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>72</v>
+        <v>78</v>
       </c>
       <c r="B4" t="s">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="D4" s="1" t="s">
         <v>64</v>
@@ -810,10 +774,10 @@
     </row>
     <row r="5" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>73</v>
+        <v>79</v>
       </c>
       <c r="B5" t="s">
-        <v>24</v>
+        <v>80</v>
       </c>
       <c r="D5" s="1" t="s">
         <v>64</v>
@@ -837,10 +801,10 @@
     </row>
     <row r="6" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>74</v>
+        <v>81</v>
       </c>
       <c r="B6" t="s">
-        <v>24</v>
+        <v>80</v>
       </c>
       <c r="D6" s="1" t="s">
         <v>64</v>
@@ -861,10 +825,10 @@
     </row>
     <row r="7" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>75</v>
+        <v>82</v>
       </c>
       <c r="B7" t="s">
-        <v>69</v>
+        <v>80</v>
       </c>
       <c r="D7" s="1" t="s">
         <v>64</v>
@@ -885,10 +849,10 @@
     </row>
     <row r="8" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>76</v>
+        <v>83</v>
       </c>
       <c r="B8" t="s">
-        <v>10</v>
+        <v>80</v>
       </c>
       <c r="D8" s="1" t="s">
         <v>64</v>
@@ -908,11 +872,11 @@
       </c>
     </row>
     <row r="9" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>77</v>
-      </c>
-      <c r="B9" t="s">
-        <v>10</v>
+      <c r="A9" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>80</v>
       </c>
       <c r="D9" s="1" t="s">
         <v>64</v>
@@ -930,11 +894,11 @@
       <c r="I9" s="1"/>
     </row>
     <row r="10" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>78</v>
-      </c>
-      <c r="B10" t="s">
-        <v>10</v>
+      <c r="A10" s="6" t="s">
+        <v>85</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>80</v>
       </c>
       <c r="D10" s="1" t="s">
         <v>64</v>
@@ -952,11 +916,11 @@
       <c r="I10" s="1"/>
     </row>
     <row r="11" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>79</v>
-      </c>
-      <c r="B11" t="s">
-        <v>16</v>
+      <c r="A11" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>87</v>
       </c>
       <c r="D11" s="1" t="s">
         <v>64</v>
@@ -974,11 +938,11 @@
       <c r="I11" s="1"/>
     </row>
     <row r="12" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>80</v>
-      </c>
-      <c r="B12" t="s">
-        <v>12</v>
+      <c r="A12" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>87</v>
       </c>
       <c r="D12" s="1" t="s">
         <v>64</v>
@@ -998,11 +962,11 @@
       </c>
     </row>
     <row r="13" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>81</v>
-      </c>
-      <c r="B13" t="s">
-        <v>12</v>
+      <c r="A13" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="B13" s="5" t="s">
+        <v>70</v>
       </c>
       <c r="D13" s="1" t="s">
         <v>64</v>
@@ -1020,11 +984,11 @@
       <c r="I13" s="1"/>
     </row>
     <row r="14" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>82</v>
-      </c>
-      <c r="B14" t="s">
-        <v>12</v>
+      <c r="A14" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="B14" s="5" t="s">
+        <v>70</v>
       </c>
       <c r="D14" s="1" t="s">
         <v>64</v>
@@ -1042,11 +1006,11 @@
       <c r="I14" s="1"/>
     </row>
     <row r="15" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>83</v>
-      </c>
-      <c r="B15" t="s">
-        <v>12</v>
+      <c r="A15" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="B15" s="5" t="s">
+        <v>70</v>
       </c>
       <c r="D15" s="1" t="s">
         <v>64</v>
@@ -1064,11 +1028,11 @@
       <c r="I15" s="1"/>
     </row>
     <row r="16" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>84</v>
-      </c>
-      <c r="B16" t="s">
-        <v>12</v>
+      <c r="A16" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="B16" s="5" t="s">
+        <v>70</v>
       </c>
       <c r="D16" s="1" t="s">
         <v>64</v>
@@ -1086,11 +1050,11 @@
       <c r="I16" s="1"/>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>85</v>
-      </c>
-      <c r="B17" t="s">
-        <v>12</v>
+      <c r="A17" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="B17" s="5" t="s">
+        <v>70</v>
       </c>
       <c r="D17" s="1" t="s">
         <v>64</v>
@@ -1108,11 +1072,11 @@
       <c r="I17" s="1"/>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
-        <v>86</v>
-      </c>
-      <c r="B18" t="s">
-        <v>10</v>
+      <c r="A18" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="B18" s="5" t="s">
+        <v>70</v>
       </c>
       <c r="D18" s="1" t="s">
         <v>64</v>
@@ -1130,11 +1094,11 @@
       <c r="I18" s="1"/>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
-        <v>87</v>
-      </c>
-      <c r="B19" t="s">
-        <v>10</v>
+      <c r="A19" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="B19" s="5" t="s">
+        <v>33</v>
       </c>
       <c r="D19" s="1" t="s">
         <v>64</v>
@@ -1154,11 +1118,11 @@
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
-        <v>88</v>
-      </c>
-      <c r="B20" t="s">
-        <v>10</v>
+      <c r="A20" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="B20" s="5" t="s">
+        <v>33</v>
       </c>
       <c r="D20" s="1" t="s">
         <v>64</v>
@@ -1178,12 +1142,6 @@
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
-        <v>89</v>
-      </c>
-      <c r="B21" t="s">
-        <v>8</v>
-      </c>
       <c r="D21" s="1" t="s">
         <v>64</v>
       </c>
@@ -1200,12 +1158,6 @@
       <c r="I21" s="1"/>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
-        <v>90</v>
-      </c>
-      <c r="B22" t="s">
-        <v>15</v>
-      </c>
       <c r="D22" s="1" t="s">
         <v>64</v>
       </c>
@@ -1224,12 +1176,8 @@
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
-        <v>91</v>
-      </c>
-      <c r="B23" t="s">
-        <v>11</v>
-      </c>
+      <c r="A23"/>
+      <c r="B23"/>
       <c r="D23" s="1" t="s">
         <v>64</v>
       </c>
@@ -1248,12 +1196,8 @@
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
-        <v>92</v>
-      </c>
-      <c r="B24" t="s">
-        <v>11</v>
-      </c>
+      <c r="A24"/>
+      <c r="B24"/>
       <c r="D24" s="1" t="s">
         <v>64</v>
       </c>
@@ -1270,12 +1214,8 @@
       <c r="I24" s="1"/>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
-        <v>93</v>
-      </c>
-      <c r="B25" t="s">
-        <v>11</v>
-      </c>
+      <c r="A25"/>
+      <c r="B25"/>
       <c r="D25" s="1" t="s">
         <v>64</v>
       </c>
@@ -1294,12 +1234,8 @@
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
-        <v>94</v>
-      </c>
-      <c r="B26" t="s">
-        <v>12</v>
-      </c>
+      <c r="A26"/>
+      <c r="B26"/>
       <c r="D26" s="1" t="s">
         <v>64</v>
       </c>
@@ -1318,12 +1254,8 @@
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
-        <v>95</v>
-      </c>
-      <c r="B27" t="s">
-        <v>12</v>
-      </c>
+      <c r="A27"/>
+      <c r="B27"/>
       <c r="D27" s="1" t="s">
         <v>64</v>
       </c>
@@ -1342,12 +1274,8 @@
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
-        <v>96</v>
-      </c>
-      <c r="B28" t="s">
-        <v>12</v>
-      </c>
+      <c r="A28"/>
+      <c r="B28"/>
       <c r="D28" s="1" t="s">
         <v>64</v>
       </c>
@@ -1364,12 +1292,8 @@
       <c r="I28" s="1"/>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A29" t="s">
-        <v>97</v>
-      </c>
-      <c r="B29" t="s">
-        <v>23</v>
-      </c>
+      <c r="A29"/>
+      <c r="B29"/>
       <c r="D29" s="1" t="s">
         <v>64</v>
       </c>
@@ -1388,12 +1312,8 @@
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A30" t="s">
-        <v>98</v>
-      </c>
-      <c r="B30" t="s">
-        <v>23</v>
-      </c>
+      <c r="A30"/>
+      <c r="B30"/>
       <c r="D30" s="1" t="s">
         <v>64</v>
       </c>
@@ -1410,12 +1330,8 @@
       <c r="I30" s="1"/>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A31" t="s">
-        <v>99</v>
-      </c>
-      <c r="B31" t="s">
-        <v>29</v>
-      </c>
+      <c r="A31"/>
+      <c r="B31"/>
       <c r="E31" s="2"/>
       <c r="G31" s="1" t="s">
         <v>4</v>
@@ -1426,12 +1342,8 @@
       <c r="I31" s="1"/>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A32" t="s">
-        <v>100</v>
-      </c>
-      <c r="B32" t="s">
-        <v>29</v>
-      </c>
+      <c r="A32"/>
+      <c r="B32"/>
       <c r="E32" s="2"/>
       <c r="G32" s="1" t="s">
         <v>4</v>
@@ -1442,20 +1354,12 @@
       <c r="I32" s="1"/>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A33" t="s">
-        <v>101</v>
-      </c>
-      <c r="B33" t="s">
-        <v>29</v>
-      </c>
+      <c r="A33"/>
+      <c r="B33"/>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A34" t="s">
-        <v>102</v>
-      </c>
-      <c r="B34" t="s">
-        <v>23</v>
-      </c>
+      <c r="A34"/>
+      <c r="B34"/>
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A44" s="6"/>
@@ -1570,42 +1474,6 @@
     </row>
     <row r="81" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A81" s="6"/>
-    </row>
-    <row r="82" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A82" s="6"/>
-    </row>
-    <row r="83" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A83" s="6"/>
-    </row>
-    <row r="84" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A84" s="6"/>
-    </row>
-    <row r="85" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A85" s="6"/>
-    </row>
-    <row r="86" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A86" s="6"/>
-    </row>
-    <row r="87" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A87" s="6"/>
-    </row>
-    <row r="88" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A88" s="6"/>
-    </row>
-    <row r="89" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A89" s="6"/>
-    </row>
-    <row r="90" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A90" s="6"/>
-    </row>
-    <row r="91" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A91" s="6"/>
-    </row>
-    <row r="92" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A92" s="6"/>
-    </row>
-    <row r="93" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A93" s="6"/>
     </row>
     <row r="94" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A94" s="6"/>
@@ -1695,28 +1563,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <Tags xmlns="c119efd6-e238-4d50-a3c0-29e100c8e97c" xsi:nil="true"/>
-    <PatchNote xmlns="c119efd6-e238-4d50-a3c0-29e100c8e97c" xsi:nil="true"/>
-    <Owner xmlns="c119efd6-e238-4d50-a3c0-29e100c8e97c" xsi:nil="true"/>
-    <FileType xmlns="c119efd6-e238-4d50-a3c0-29e100c8e97c" xsi:nil="true"/>
-    <ProjectName xmlns="c119efd6-e238-4d50-a3c0-29e100c8e97c" xsi:nil="true"/>
-    <ShortDescription xmlns="c119efd6-e238-4d50-a3c0-29e100c8e97c" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100C661DF1982CF5C45AD6C977DF31A5F9E" ma:contentTypeVersion="10" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="9bea797a5b2c9e3b07e1ad7cf473c08b">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="c119efd6-e238-4d50-a3c0-29e100c8e97c" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="bd93c1d0aea623e2b9aecd5ac10b5033" ns2:_="">
     <xsd:import namespace="c119efd6-e238-4d50-a3c0-29e100c8e97c"/>
@@ -1906,25 +1752,29 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{99A9B5FE-848A-4976-BAAE-EC968E54ED3B}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="c119efd6-e238-4d50-a3c0-29e100c8e97c"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <Tags xmlns="c119efd6-e238-4d50-a3c0-29e100c8e97c" xsi:nil="true"/>
+    <PatchNote xmlns="c119efd6-e238-4d50-a3c0-29e100c8e97c" xsi:nil="true"/>
+    <Owner xmlns="c119efd6-e238-4d50-a3c0-29e100c8e97c" xsi:nil="true"/>
+    <FileType xmlns="c119efd6-e238-4d50-a3c0-29e100c8e97c" xsi:nil="true"/>
+    <ProjectName xmlns="c119efd6-e238-4d50-a3c0-29e100c8e97c" xsi:nil="true"/>
+    <ShortDescription xmlns="c119efd6-e238-4d50-a3c0-29e100c8e97c" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4D936FB1-25F6-4ACA-A9FB-DBC1D231A01B}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6427767B-DBAA-499C-AB6C-5A5080D50FBD}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1940,4 +1790,22 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{99A9B5FE-848A-4976-BAAE-EC968E54ED3B}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="c119efd6-e238-4d50-a3c0-29e100c8e97c"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4D936FB1-25F6-4ACA-A9FB-DBC1D231A01B}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
25 Aug 2026 - Upgrade to 26C
</commit_message>
<xml_diff>
--- a/Import_WD.xlsx
+++ b/Import_WD.xlsx
@@ -1,42 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ichorsystems-my.sharepoint.com/personal/kmageshkumar_ichorsystems_com/Documents/Scripts/WD Create FBDI/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="118" documentId="13_ncr:1_{1448A942-2B91-453D-A348-8841A73FF17B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{17C8CA57-6B38-4222-A65B-58993127ABE4}"/>
+  <xr:revisionPtr revIDLastSave="25" documentId="11_F85AFEDEC97FC7717684D3E7F316E641423A3527" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2DA246C5-63BB-4DFF-A42D-4728F98F5A06}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="182" uniqueCount="91">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="172" uniqueCount="83">
   <si>
     <t>WD Number</t>
   </si>
@@ -44,102 +28,198 @@
     <t>Template to use (List of Templates is on the right)</t>
   </si>
   <si>
+    <t>Customer</t>
+  </si>
+  <si>
     <t>WD Templates</t>
   </si>
   <si>
-    <t>Customer</t>
+    <t>Verified to be working (Temp)</t>
+  </si>
+  <si>
+    <t>SGP_TEMPLATE_LAM_EOS_DA_ESX</t>
+  </si>
+  <si>
+    <t>LAM</t>
+  </si>
+  <si>
+    <t>SGP_TEMPLATE_LAM_GB_JTS</t>
   </si>
   <si>
     <t>AMAT</t>
   </si>
   <si>
-    <t>SGP_TEMPLATE_LAM_GB_JTS</t>
-  </si>
-  <si>
     <t>SGP_TEMPLATE_AMAT_INZC_1</t>
   </si>
   <si>
+    <t>Y</t>
+  </si>
+  <si>
+    <t>SGP_TEMPLATE_LAM_EOS_DA_DSL</t>
+  </si>
+  <si>
     <t>SGP_TEMPLATE_AMAT_INZC_2</t>
   </si>
   <si>
     <t>SGP_TEMPLATE_AMAT_INZC_3</t>
   </si>
   <si>
+    <t>SGP_TEMPLATE_LAM_EOS_INTCON</t>
+  </si>
+  <si>
     <t>SGP_TEMPLATE_AMAT_GT_GPLIS</t>
   </si>
   <si>
+    <t xml:space="preserve"> </t>
+  </si>
+  <si>
+    <t>SGP_TEMPLATE_LAM_EOS_GB</t>
+  </si>
+  <si>
+    <t>SGP_TEMPLATE_LAM_EOS_DA_MOD</t>
+  </si>
+  <si>
     <t>SGP_TEMPLATE_AMAT_GT</t>
   </si>
   <si>
+    <t>SGP_TEMPLATE_LAM_UFA_E4</t>
+  </si>
+  <si>
     <t>SGP_AMAT_SE_1_CH_GPLIS</t>
   </si>
   <si>
+    <t>SGP_TEMPLATE_LAM_UFA_E5</t>
+  </si>
+  <si>
     <t>SGP_AMAT_SE_1_CH</t>
   </si>
   <si>
+    <t>SGP_TEMPLATE_LAM_UFA_E6</t>
+  </si>
+  <si>
     <t>SGP_AMAT_SE_2_CH_GPLIS</t>
   </si>
   <si>
+    <t>SGP_TEMPLATE_LAM_UFA_KIT</t>
+  </si>
+  <si>
     <t>SGP_AMAT_SE_2_CH</t>
   </si>
   <si>
+    <t>SGP_TEMPLATE_LAM_GB_IGS</t>
+  </si>
+  <si>
     <t>SGP_AMAT_SE_3_CH_GPLIS</t>
   </si>
   <si>
     <t>SGP_AMAT_SE_3_CH</t>
   </si>
   <si>
+    <t>SGP_TEMPLATE_LAM_GB_JTS_KIT</t>
+  </si>
+  <si>
     <t>SGP_TEMPLATE_AMAT_SE_FRAME</t>
   </si>
   <si>
+    <t>SGP_TEMPLATE_LAM_GB_JTS2</t>
+  </si>
+  <si>
     <t>SGP_TEMPLATE_AMAT_SE_UV</t>
   </si>
   <si>
+    <t>SGP_TEMPLATE_LAM_GB_JTS2_KIT</t>
+  </si>
+  <si>
     <t>SGP_TEMPLATE_AMAT_NEXTGEN_1</t>
   </si>
   <si>
+    <t>SGP_TEMPLATE_LAM_ICS</t>
+  </si>
+  <si>
     <t>SGP_TEMPLATE_AMAT_NEXTGEN_2</t>
   </si>
   <si>
+    <t>SGP_TEMPLATE_LAM_ZONE</t>
+  </si>
+  <si>
     <t>SGP_TEMPLATE_AMAT_NEXTGEN_3</t>
   </si>
   <si>
+    <t>SGP_TEMPLATE_LAM_SENSEI_FIP</t>
+  </si>
+  <si>
     <t>SGP_TEMPLATE_AMAT_NEXTGEN_4</t>
   </si>
   <si>
+    <t>SGP_TEMPLATE_LAM_SENSEI_BRIDGE</t>
+  </si>
+  <si>
     <t>SGP_TEMPLATE_AMAT_NEXTGEN_SLD</t>
   </si>
   <si>
+    <t>SGP_TEMPLATE_LAM_SENSEI_FIB</t>
+  </si>
+  <si>
     <t>SGP_TEMPLATE_AMAT_APACHE</t>
   </si>
   <si>
+    <t>SGP_TEMPLATE_LAM_SENSEI_PF_L6</t>
+  </si>
+  <si>
     <t>SGP_TEMPLATE_AMAT_APACHE_GPLIS</t>
   </si>
   <si>
+    <t>SGP_TEMPLATE_LAM_ARGOS</t>
+  </si>
+  <si>
     <t>SGP_TEMPLATE_AMAT_JOPLIN</t>
   </si>
   <si>
+    <t>SGP_TEMPLATE_LAM_MOBI</t>
+  </si>
+  <si>
     <t>SGP_TEMPLATE_AMAT_JOPLIN_LDS</t>
   </si>
   <si>
+    <t>SGP_TEMPLATE_LAM_NPI</t>
+  </si>
+  <si>
     <t>SGP_TEMPLATE_AMAT_ERMIAS</t>
   </si>
   <si>
+    <t>SGP_TEMPLATE_LAM_AFVI_GB</t>
+  </si>
+  <si>
     <t>SGP_TEMPLATE_AMAT_SYM3</t>
   </si>
   <si>
+    <t>SGP_TEMPLATE_LAM_AFVI2_GB_SINGLE</t>
+  </si>
+  <si>
     <t>SGP_TEMPLATE_AMAT_SICONI_OATES</t>
   </si>
   <si>
+    <t>SGP_TEMPLATE_LAM_AFVI2_GB_DUAL</t>
+  </si>
+  <si>
     <t>SGP_TEMPLATE_AMAT_TXZ</t>
   </si>
   <si>
+    <t>SGP_TEMPLATE_LAM_AFVI_GB_SO</t>
+  </si>
+  <si>
     <t>SGP_TEMPLATE_AMAT_GPLL</t>
   </si>
   <si>
+    <t>SGP_TEMPLATE_LAM_EOS_DA_KIT</t>
+  </si>
+  <si>
     <t>SGP_TEMPLATE_AMAT_EPI</t>
   </si>
   <si>
+    <t>SGP_TEMPLATE_LAM_AFVI2_JTS</t>
+  </si>
+  <si>
     <t>SGP_AMAT_APACHE_NSO_S</t>
   </si>
   <si>
@@ -149,166 +229,46 @@
     <t>SGP_AMAT_CLARION2</t>
   </si>
   <si>
-    <t xml:space="preserve"> </t>
-  </si>
-  <si>
-    <t>Verified to be working (Temp)</t>
-  </si>
-  <si>
-    <t>SGP_TEMPLATE_LAM_EOS_GB</t>
-  </si>
-  <si>
-    <t>SGP_TEMPLATE_LAM_EOS_DA_DSL</t>
-  </si>
-  <si>
-    <t>SGP_TEMPLATE_LAM_EOS_DA_ESX</t>
-  </si>
-  <si>
-    <t>SGP_TEMPLATE_LAM_EOS_INTCON</t>
-  </si>
-  <si>
-    <t>SGP_TEMPLATE_LAM_EOS_DA_MOD</t>
-  </si>
-  <si>
-    <t>SGP_TEMPLATE_LAM_UFA_E4</t>
-  </si>
-  <si>
-    <t>SGP_TEMPLATE_LAM_UFA_E5</t>
-  </si>
-  <si>
-    <t>SGP_TEMPLATE_LAM_UFA_E6</t>
-  </si>
-  <si>
-    <t>SGP_TEMPLATE_LAM_UFA_KIT</t>
-  </si>
-  <si>
-    <t>SGP_TEMPLATE_LAM_GB_IGS</t>
-  </si>
-  <si>
-    <t>SGP_TEMPLATE_LAM_GB_JTS_KIT</t>
-  </si>
-  <si>
-    <t>SGP_TEMPLATE_LAM_GB_JTS2</t>
-  </si>
-  <si>
-    <t>SGP_TEMPLATE_LAM_GB_JTS2_KIT</t>
-  </si>
-  <si>
-    <t>SGP_TEMPLATE_LAM_ICS</t>
-  </si>
-  <si>
-    <t>SGP_TEMPLATE_LAM_ZONE</t>
-  </si>
-  <si>
-    <t>SGP_TEMPLATE_LAM_SENSEI_FIP</t>
-  </si>
-  <si>
-    <t>SGP_TEMPLATE_LAM_SENSEI_BRIDGE</t>
-  </si>
-  <si>
-    <t>SGP_TEMPLATE_LAM_SENSEI_FIB</t>
-  </si>
-  <si>
-    <t>SGP_TEMPLATE_LAM_SENSEI_PF_L6</t>
-  </si>
-  <si>
-    <t>SGP_TEMPLATE_LAM_ARGOS</t>
-  </si>
-  <si>
-    <t>SGP_TEMPLATE_LAM_MOBI</t>
-  </si>
-  <si>
-    <t>SGP_TEMPLATE_LAM_NPI</t>
-  </si>
-  <si>
-    <t>SGP_TEMPLATE_LAM_AFVI_GB</t>
-  </si>
-  <si>
-    <t>SGP_TEMPLATE_LAM_AFVI2_GB_SINGLE</t>
-  </si>
-  <si>
-    <t>SGP_TEMPLATE_LAM_AFVI2_GB_DUAL</t>
-  </si>
-  <si>
-    <t>LAM</t>
-  </si>
-  <si>
-    <t>Y</t>
-  </si>
-  <si>
-    <t>SGP_TEMPLATE_LAM_AFVI_GB_SO</t>
-  </si>
-  <si>
-    <t>SGP_TEMPLATE_LAM_EOS_DA_KIT</t>
-  </si>
-  <si>
-    <t>SGP_TEMPLATE_LAM_AFVI2_JTS</t>
-  </si>
-  <si>
-    <t>A04027-TY-GPA</t>
-  </si>
-  <si>
-    <t>SGP_TEMPLATE_DPN</t>
-  </si>
-  <si>
-    <t>A04027-TY-GPB</t>
-  </si>
-  <si>
-    <t>A04622-TY-GPC</t>
-  </si>
-  <si>
-    <t>A04622-TY-GPD</t>
-  </si>
-  <si>
-    <t>A04619-TY-GPA</t>
-  </si>
-  <si>
-    <t>A04619-TY-GPB</t>
-  </si>
-  <si>
-    <t>709850-XA3T-GPA</t>
-  </si>
-  <si>
-    <t>709850-XA3T-GPB</t>
-  </si>
-  <si>
-    <t>709850-XA3T-GPC</t>
-  </si>
-  <si>
-    <t>710366-XXT-GPA</t>
-  </si>
-  <si>
-    <t>SGP_TEMPLATE_NAPA</t>
-  </si>
-  <si>
-    <t>710366-XXT-GPB</t>
-  </si>
-  <si>
-    <t>710366-XXT-GPC</t>
-  </si>
-  <si>
-    <t>710411-XXT-GPA</t>
-  </si>
-  <si>
-    <t>710411-XXT-GPB</t>
-  </si>
-  <si>
-    <t>710411-XXT-GPC</t>
-  </si>
-  <si>
-    <t>A02651R2-TY-GPA</t>
-  </si>
-  <si>
-    <t>SGP_TEMPLATE_NSO_1_STICK</t>
-  </si>
-  <si>
-    <t>A02651R2-TY-GPD</t>
-  </si>
-  <si>
-    <t>C02371-EY2-GP1</t>
-  </si>
-  <si>
-    <t>C02371-EY2-GP2</t>
+    <t>709831-XA2-GP</t>
+  </si>
+  <si>
+    <t>C02053-EY3-GP2A</t>
+  </si>
+  <si>
+    <t>C02053-EY3-GP2B</t>
+  </si>
+  <si>
+    <t>C02053-EY3-GP2C</t>
+  </si>
+  <si>
+    <t>C02053-EY3-GP2D</t>
+  </si>
+  <si>
+    <t>C02151-EY3-GP2A</t>
+  </si>
+  <si>
+    <t>C02151-EY3-GP2B</t>
+  </si>
+  <si>
+    <t>C02151-EY3-GP2C</t>
+  </si>
+  <si>
+    <t>C02151-EY3-GP2D</t>
+  </si>
+  <si>
+    <t>C02283-EY3-GPA</t>
+  </si>
+  <si>
+    <t>C02283-EY3-GPB</t>
+  </si>
+  <si>
+    <t>C02283-EY3-GPC</t>
+  </si>
+  <si>
+    <t>C02480-EY1-GP1</t>
+  </si>
+  <si>
+    <t>C02480-EY1-GP2</t>
   </si>
 </sst>
 </file>
@@ -684,696 +644,644 @@
         <v>1</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="H1" s="1" t="s">
-        <v>2</v>
-      </c>
       <c r="I1" s="1" t="s">
-        <v>38</v>
+        <v>4</v>
       </c>
     </row>
     <row r="2" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>76</v>
+        <v>69</v>
       </c>
       <c r="B2" t="s">
-        <v>29</v>
+        <v>42</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>64</v>
+        <v>6</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="F2" s="1"/>
       <c r="G2" s="1" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="H2" s="4" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>65</v>
+        <v>10</v>
       </c>
     </row>
     <row r="3" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>77</v>
+        <v>70</v>
       </c>
       <c r="B3" t="s">
-        <v>29</v>
+        <v>50</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>64</v>
+        <v>6</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>40</v>
+        <v>11</v>
       </c>
       <c r="F3" s="1"/>
       <c r="G3" s="1" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="H3" s="4" t="s">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="I3" s="1"/>
     </row>
     <row r="4" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>78</v>
+        <v>71</v>
       </c>
       <c r="B4" t="s">
-        <v>29</v>
+        <v>50</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>64</v>
+        <v>6</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>41</v>
+        <v>5</v>
       </c>
       <c r="F4" s="1"/>
       <c r="G4" s="1" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="I4" s="1" t="s">
-        <v>65</v>
+        <v>10</v>
       </c>
     </row>
     <row r="5" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>79</v>
+        <v>72</v>
       </c>
       <c r="B5" t="s">
-        <v>80</v>
+        <v>50</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>64</v>
+        <v>6</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>42</v>
+        <v>14</v>
       </c>
       <c r="F5" s="1"/>
       <c r="G5" s="1" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="H5" s="4" t="s">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="I5" s="1" t="s">
-        <v>65</v>
+        <v>10</v>
       </c>
       <c r="R5" t="s">
-        <v>37</v>
+        <v>16</v>
       </c>
     </row>
     <row r="6" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>81</v>
+      <c r="A6" s="6" t="s">
+        <v>73</v>
       </c>
       <c r="B6" t="s">
-        <v>80</v>
+        <v>50</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>64</v>
+        <v>6</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>43</v>
+        <v>18</v>
       </c>
       <c r="F6" s="1"/>
       <c r="G6" s="1" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="H6" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="I6" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="I6" s="1" t="s">
-        <v>65</v>
-      </c>
     </row>
     <row r="7" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>82</v>
+      <c r="A7" s="6" t="s">
+        <v>74</v>
       </c>
       <c r="B7" t="s">
-        <v>80</v>
+        <v>50</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>64</v>
+        <v>6</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>44</v>
+        <v>20</v>
       </c>
       <c r="F7" s="1"/>
       <c r="G7" s="1" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="H7" s="4" t="s">
-        <v>11</v>
+        <v>21</v>
       </c>
       <c r="I7" s="1" t="s">
-        <v>65</v>
+        <v>10</v>
       </c>
     </row>
     <row r="8" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>83</v>
+      <c r="A8" s="6" t="s">
+        <v>75</v>
       </c>
       <c r="B8" t="s">
-        <v>80</v>
+        <v>50</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>64</v>
+        <v>6</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>45</v>
+        <v>22</v>
       </c>
       <c r="F8" s="1"/>
       <c r="G8" s="1" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="H8" s="4" t="s">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="I8" s="1" t="s">
-        <v>65</v>
+        <v>10</v>
       </c>
     </row>
     <row r="9" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A9" s="6" t="s">
-        <v>84</v>
-      </c>
-      <c r="B9" s="5" t="s">
-        <v>80</v>
+      <c r="A9" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="B9" t="s">
+        <v>50</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>64</v>
+        <v>6</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>46</v>
+        <v>24</v>
       </c>
       <c r="F9" s="1"/>
       <c r="G9" s="1" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="H9" s="4" t="s">
-        <v>13</v>
+        <v>25</v>
       </c>
       <c r="I9" s="1"/>
     </row>
     <row r="10" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A10" s="6" t="s">
-        <v>85</v>
-      </c>
-      <c r="B10" s="5" t="s">
-        <v>80</v>
+      <c r="A10" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="B10" t="s">
+        <v>50</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>64</v>
+        <v>6</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>47</v>
+        <v>26</v>
       </c>
       <c r="F10" s="1"/>
       <c r="G10" s="1" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="H10" s="4" t="s">
-        <v>14</v>
+        <v>27</v>
       </c>
       <c r="I10" s="1"/>
     </row>
     <row r="11" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A11" s="6" t="s">
-        <v>86</v>
-      </c>
-      <c r="B11" s="5" t="s">
-        <v>87</v>
+      <c r="A11" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="B11" t="s">
+        <v>50</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>64</v>
+        <v>6</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>48</v>
+        <v>28</v>
       </c>
       <c r="F11" s="1"/>
       <c r="G11" s="1" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="H11" s="4" t="s">
-        <v>15</v>
+        <v>29</v>
       </c>
       <c r="I11" s="1"/>
     </row>
     <row r="12" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>87</v>
+        <v>50</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>64</v>
+        <v>6</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>39</v>
+        <v>17</v>
       </c>
       <c r="F12" s="1"/>
       <c r="G12" s="1" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="H12" s="4" t="s">
-        <v>16</v>
+        <v>30</v>
       </c>
       <c r="I12" s="1" t="s">
-        <v>65</v>
+        <v>10</v>
       </c>
     </row>
     <row r="13" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
-        <v>69</v>
+        <v>80</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>70</v>
+        <v>50</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>64</v>
+        <v>6</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>49</v>
+        <v>31</v>
       </c>
       <c r="F13" s="1"/>
       <c r="G13" s="1" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="H13" s="4" t="s">
-        <v>17</v>
+        <v>32</v>
       </c>
       <c r="I13" s="1"/>
     </row>
     <row r="14" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A14" s="5" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>64</v>
+        <v>6</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>50</v>
+        <v>33</v>
       </c>
       <c r="F14" s="1"/>
       <c r="G14" s="1" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="H14" s="4" t="s">
-        <v>18</v>
+        <v>34</v>
       </c>
       <c r="I14" s="1"/>
     </row>
     <row r="15" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A15" s="5" t="s">
-        <v>74</v>
+        <v>82</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>64</v>
+        <v>6</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>51</v>
+        <v>35</v>
       </c>
       <c r="F15" s="1"/>
       <c r="G15" s="1" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="H15" s="4" t="s">
-        <v>19</v>
+        <v>36</v>
       </c>
       <c r="I15" s="1"/>
     </row>
     <row r="16" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A16" s="5" t="s">
-        <v>75</v>
-      </c>
-      <c r="B16" s="5" t="s">
-        <v>70</v>
-      </c>
       <c r="D16" s="1" t="s">
-        <v>64</v>
+        <v>6</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>52</v>
+        <v>37</v>
       </c>
       <c r="F16" s="1"/>
       <c r="G16" s="1" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="H16" s="4" t="s">
-        <v>20</v>
+        <v>38</v>
       </c>
       <c r="I16" s="1"/>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A17" s="5" t="s">
-        <v>72</v>
-      </c>
-      <c r="B17" s="5" t="s">
-        <v>70</v>
-      </c>
+    <row r="17" spans="4:9" x14ac:dyDescent="0.25">
       <c r="D17" s="1" t="s">
-        <v>64</v>
+        <v>6</v>
       </c>
       <c r="E17" s="3" t="s">
-        <v>53</v>
+        <v>39</v>
       </c>
       <c r="F17" s="1"/>
       <c r="G17" s="1" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="H17" s="4" t="s">
-        <v>21</v>
+        <v>40</v>
       </c>
       <c r="I17" s="1"/>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A18" s="5" t="s">
-        <v>73</v>
-      </c>
-      <c r="B18" s="5" t="s">
-        <v>70</v>
-      </c>
+    <row r="18" spans="4:9" x14ac:dyDescent="0.25">
       <c r="D18" s="1" t="s">
-        <v>64</v>
+        <v>6</v>
       </c>
       <c r="E18" s="3" t="s">
-        <v>54</v>
+        <v>41</v>
       </c>
       <c r="F18" s="1"/>
       <c r="G18" s="1" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="H18" s="4" t="s">
-        <v>22</v>
+        <v>42</v>
       </c>
       <c r="I18" s="1"/>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A19" s="5" t="s">
-        <v>89</v>
-      </c>
-      <c r="B19" s="5" t="s">
-        <v>33</v>
-      </c>
+    <row r="19" spans="4:9" x14ac:dyDescent="0.25">
       <c r="D19" s="1" t="s">
-        <v>64</v>
+        <v>6</v>
       </c>
       <c r="E19" s="3" t="s">
-        <v>55</v>
+        <v>43</v>
       </c>
       <c r="F19" s="1"/>
       <c r="G19" s="1" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="H19" s="4" t="s">
-        <v>23</v>
+        <v>44</v>
       </c>
       <c r="I19" s="1" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A20" s="5" t="s">
-        <v>90</v>
-      </c>
-      <c r="B20" s="5" t="s">
-        <v>33</v>
-      </c>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="20" spans="4:9" x14ac:dyDescent="0.25">
       <c r="D20" s="1" t="s">
-        <v>64</v>
+        <v>6</v>
       </c>
       <c r="E20" s="3" t="s">
-        <v>56</v>
+        <v>45</v>
       </c>
       <c r="F20" s="1"/>
       <c r="G20" s="1" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="H20" s="4" t="s">
-        <v>24</v>
+        <v>46</v>
       </c>
       <c r="I20" s="1" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="21" spans="4:9" x14ac:dyDescent="0.25">
       <c r="D21" s="1" t="s">
-        <v>64</v>
+        <v>6</v>
       </c>
       <c r="E21" s="3" t="s">
-        <v>57</v>
+        <v>47</v>
       </c>
       <c r="F21" s="1"/>
       <c r="G21" s="1" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="H21" s="4" t="s">
-        <v>25</v>
+        <v>48</v>
       </c>
       <c r="I21" s="1"/>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="22" spans="4:9" x14ac:dyDescent="0.25">
       <c r="D22" s="1" t="s">
-        <v>64</v>
+        <v>6</v>
       </c>
       <c r="E22" s="3" t="s">
-        <v>58</v>
+        <v>49</v>
       </c>
       <c r="F22" s="1"/>
       <c r="G22" s="1" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="H22" s="4" t="s">
-        <v>26</v>
+        <v>50</v>
       </c>
       <c r="I22" s="1" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A23"/>
-      <c r="B23"/>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="23" spans="4:9" x14ac:dyDescent="0.25">
       <c r="D23" s="1" t="s">
-        <v>64</v>
+        <v>6</v>
       </c>
       <c r="E23" s="3" t="s">
-        <v>59</v>
+        <v>51</v>
       </c>
       <c r="F23" s="1"/>
       <c r="G23" s="1" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="H23" s="4" t="s">
-        <v>27</v>
+        <v>52</v>
       </c>
       <c r="I23" s="1" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A24"/>
-      <c r="B24"/>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="24" spans="4:9" x14ac:dyDescent="0.25">
       <c r="D24" s="1" t="s">
-        <v>64</v>
+        <v>6</v>
       </c>
       <c r="E24" s="3" t="s">
-        <v>60</v>
+        <v>53</v>
       </c>
       <c r="F24" s="1"/>
       <c r="G24" s="1" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="H24" s="4" t="s">
-        <v>28</v>
+        <v>54</v>
       </c>
       <c r="I24" s="1"/>
     </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A25"/>
-      <c r="B25"/>
+    <row r="25" spans="4:9" x14ac:dyDescent="0.25">
       <c r="D25" s="1" t="s">
-        <v>64</v>
+        <v>6</v>
       </c>
       <c r="E25" s="3" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
       <c r="F25" s="1"/>
       <c r="G25" s="1" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="H25" s="4" t="s">
-        <v>29</v>
+        <v>56</v>
       </c>
       <c r="I25" s="1" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A26"/>
-      <c r="B26"/>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="26" spans="4:9" x14ac:dyDescent="0.25">
       <c r="D26" s="1" t="s">
-        <v>64</v>
+        <v>6</v>
       </c>
       <c r="E26" s="3" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="F26" s="1"/>
       <c r="G26" s="1" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="H26" s="4" t="s">
-        <v>30</v>
+        <v>58</v>
       </c>
       <c r="I26" s="1" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A27"/>
-      <c r="B27"/>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="27" spans="4:9" x14ac:dyDescent="0.25">
       <c r="D27" s="1" t="s">
-        <v>64</v>
+        <v>6</v>
       </c>
       <c r="E27" s="3" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="F27" s="1"/>
       <c r="G27" s="1" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="H27" s="4" t="s">
-        <v>31</v>
+        <v>60</v>
       </c>
       <c r="I27" s="1" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A28"/>
-      <c r="B28"/>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="28" spans="4:9" x14ac:dyDescent="0.25">
       <c r="D28" s="1" t="s">
-        <v>64</v>
+        <v>6</v>
       </c>
       <c r="E28" s="4" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="F28" s="1"/>
       <c r="G28" s="1" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="H28" s="4" t="s">
-        <v>32</v>
+        <v>62</v>
       </c>
       <c r="I28" s="1"/>
     </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A29"/>
-      <c r="B29"/>
+    <row r="29" spans="4:9" x14ac:dyDescent="0.25">
       <c r="D29" s="1" t="s">
-        <v>64</v>
+        <v>6</v>
       </c>
       <c r="E29" s="4" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="F29" s="1"/>
       <c r="G29" s="1" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="H29" s="4" t="s">
-        <v>33</v>
+        <v>64</v>
       </c>
       <c r="I29" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="30" spans="4:9" x14ac:dyDescent="0.25">
+      <c r="D30" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E30" s="4" t="s">
         <v>65</v>
-      </c>
-    </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A30"/>
-      <c r="B30"/>
-      <c r="D30" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="E30" s="4" t="s">
-        <v>68</v>
       </c>
       <c r="F30" s="1"/>
       <c r="G30" s="1" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="H30" s="3" t="s">
-        <v>34</v>
+        <v>66</v>
       </c>
       <c r="I30" s="1"/>
     </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A31"/>
-      <c r="B31"/>
+    <row r="31" spans="4:9" x14ac:dyDescent="0.25">
       <c r="E31" s="2"/>
       <c r="G31" s="1" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="H31" s="3" t="s">
-        <v>35</v>
+        <v>67</v>
       </c>
       <c r="I31" s="1"/>
     </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A32"/>
-      <c r="B32"/>
+    <row r="32" spans="4:9" x14ac:dyDescent="0.25">
       <c r="E32" s="2"/>
       <c r="G32" s="1" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="H32" s="3" t="s">
-        <v>36</v>
+        <v>68</v>
       </c>
       <c r="I32" s="1"/>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A33"/>
-      <c r="B33"/>
-    </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A34"/>
-      <c r="B34"/>
-    </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A42" s="6"/>
+    </row>
+    <row r="43" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A43" s="6"/>
+    </row>
+    <row r="44" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A44" s="6"/>
     </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A45" s="6"/>
     </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A46" s="6"/>
     </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A47" s="6"/>
     </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A48" s="6"/>
     </row>
     <row r="49" spans="1:1" x14ac:dyDescent="0.25">
@@ -1412,12 +1320,6 @@
     <row r="60" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A60" s="6"/>
     </row>
-    <row r="61" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A61" s="6"/>
-    </row>
-    <row r="62" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A62" s="6"/>
-    </row>
     <row r="63" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A63" s="6"/>
     </row>
@@ -1558,254 +1460,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait"/>
 </worksheet>
-</file>
-
-<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100C661DF1982CF5C45AD6C977DF31A5F9E" ma:contentTypeVersion="10" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="9bea797a5b2c9e3b07e1ad7cf473c08b">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="c119efd6-e238-4d50-a3c0-29e100c8e97c" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="bd93c1d0aea623e2b9aecd5ac10b5033" ns2:_="">
-    <xsd:import namespace="c119efd6-e238-4d50-a3c0-29e100c8e97c"/>
-    <xsd:element name="properties">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element name="documentManagement">
-            <xsd:complexType>
-              <xsd:all>
-                <xsd:element ref="ns2:FileType" minOccurs="0"/>
-                <xsd:element ref="ns2:Tags" minOccurs="0"/>
-                <xsd:element ref="ns2:ShortDescription" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
-                <xsd:element ref="ns2:ProjectName" minOccurs="0"/>
-                <xsd:element ref="ns2:Owner" minOccurs="0"/>
-                <xsd:element ref="ns2:PatchNote" minOccurs="0"/>
-              </xsd:all>
-            </xsd:complexType>
-          </xsd:element>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="c119efd6-e238-4d50-a3c0-29e100c8e97c" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="FileType" ma:index="8" nillable="true" ma:displayName="FileType" ma:description="Type of content" ma:format="Dropdown" ma:internalName="FileType">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Choice">
-          <xsd:enumeration value="Python Script"/>
-          <xsd:enumeration value="Excel Macro"/>
-          <xsd:enumeration value="Readme"/>
-          <xsd:enumeration value="Folder"/>
-          <xsd:enumeration value="Dependent File"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="Tags" ma:index="9" nillable="true" ma:displayName="Tags" ma:description="Searchable tags for future queries, for example: Agile, ECO, Download" ma:format="Dropdown" ma:internalName="Tags">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="ShortDescription" ma:index="10" nillable="true" ma:displayName="Short Description" ma:description="Short Description" ma:format="Dropdown" ma:internalName="ShortDescription">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="ProjectName" ma:index="14" nillable="true" ma:displayName="Project Name" ma:description="Groups files that are needed in the same project" ma:format="Dropdown" ma:internalName="ProjectName">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="Owner" ma:index="15" nillable="true" ma:displayName="Owner" ma:format="Dropdown" ma:internalName="Owner">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Choice">
-          <xsd:enumeration value="Ivan"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="PatchNote" ma:index="16" nillable="true" ma:displayName="Patch Notes" ma:format="Dropdown" ma:internalName="PatchNote">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
-    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
-    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
-    <xsd:element name="coreProperties" type="CT_coreProperties"/>
-    <xsd:complexType name="CT_coreProperties">
-      <xsd:all>
-        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
-        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
-        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
-          <xsd:annotation>
-            <xsd:documentation>
-                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
-                    </xsd:documentation>
-          </xsd:annotation>
-        </xsd:element>
-        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-      </xsd:all>
-    </xsd:complexType>
-  </xsd:schema>
-  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
-    <xs:element name="Person">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:DisplayName" minOccurs="0"/>
-          <xs:element ref="pc:AccountId" minOccurs="0"/>
-          <xs:element ref="pc:AccountType" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="DisplayName" type="xs:string"/>
-    <xs:element name="AccountId" type="xs:string"/>
-    <xs:element name="AccountType" type="xs:string"/>
-    <xs:element name="BDCAssociatedEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-        <xs:attribute ref="pc:EntityNamespace"/>
-        <xs:attribute ref="pc:EntityName"/>
-        <xs:attribute ref="pc:SystemInstanceName"/>
-        <xs:attribute ref="pc:AssociationName"/>
-      </xs:complexType>
-    </xs:element>
-    <xs:attribute name="EntityNamespace" type="xs:string"/>
-    <xs:attribute name="EntityName" type="xs:string"/>
-    <xs:attribute name="SystemInstanceName" type="xs:string"/>
-    <xs:attribute name="AssociationName" type="xs:string"/>
-    <xs:element name="BDCEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
-          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
-          <xs:element ref="pc:EntityId1" minOccurs="0"/>
-          <xs:element ref="pc:EntityId2" minOccurs="0"/>
-          <xs:element ref="pc:EntityId3" minOccurs="0"/>
-          <xs:element ref="pc:EntityId4" minOccurs="0"/>
-          <xs:element ref="pc:EntityId5" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="EntityDisplayName" type="xs:string"/>
-    <xs:element name="EntityInstanceReference" type="xs:string"/>
-    <xs:element name="EntityId1" type="xs:string"/>
-    <xs:element name="EntityId2" type="xs:string"/>
-    <xs:element name="EntityId3" type="xs:string"/>
-    <xs:element name="EntityId4" type="xs:string"/>
-    <xs:element name="EntityId5" type="xs:string"/>
-    <xs:element name="Terms">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermInfo">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermName" minOccurs="0"/>
-          <xs:element ref="pc:TermId" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermName" type="xs:string"/>
-    <xs:element name="TermId" type="xs:string"/>
-  </xs:schema>
-</ct:contentTypeSchema>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <Tags xmlns="c119efd6-e238-4d50-a3c0-29e100c8e97c" xsi:nil="true"/>
-    <PatchNote xmlns="c119efd6-e238-4d50-a3c0-29e100c8e97c" xsi:nil="true"/>
-    <Owner xmlns="c119efd6-e238-4d50-a3c0-29e100c8e97c" xsi:nil="true"/>
-    <FileType xmlns="c119efd6-e238-4d50-a3c0-29e100c8e97c" xsi:nil="true"/>
-    <ProjectName xmlns="c119efd6-e238-4d50-a3c0-29e100c8e97c" xsi:nil="true"/>
-    <ShortDescription xmlns="c119efd6-e238-4d50-a3c0-29e100c8e97c" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6427767B-DBAA-499C-AB6C-5A5080D50FBD}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="c119efd6-e238-4d50-a3c0-29e100c8e97c"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{99A9B5FE-848A-4976-BAAE-EC968E54ED3B}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="c119efd6-e238-4d50-a3c0-29e100c8e97c"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4D936FB1-25F6-4ACA-A9FB-DBC1D231A01B}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>